<commit_message>
Regenerate data.js from Robot_model.xlsx and Robot_spec.xlsx with updated models and specs
</commit_message>
<xml_diff>
--- a/InoRobotSelect/Robot_spec.xlsx
+++ b/InoRobotSelect/Robot_spec.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b96646d0fc390357/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b96646d0fc390357/Desktop/made_C^N/InoRobotAssistant/InoRobotSelect/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="309" documentId="8_{522FA3AE-843B-45F5-9EBE-713FE4E8C55E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{733BA37F-26CD-4422-9157-FC2B0F46A7BC}"/>
+  <xr:revisionPtr revIDLastSave="323" documentId="8_{522FA3AE-843B-45F5-9EBE-713FE4E8C55E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E12D8BA1-58AD-432E-AC83-292119DE4DDD}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{166C1812-565C-44F3-A85A-A23A1F110762}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1169" uniqueCount="329">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1209" uniqueCount="330">
   <si>
     <t>Spec / Model</t>
   </si>
@@ -1136,6 +1136,10 @@
   </si>
   <si>
     <t>Stand:3m Option:5/10/15m</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>IP20</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
@@ -1858,7 +1862,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1910,7 +1914,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1925,16 +1929,10 @@
     <xf numFmtId="0" fontId="23" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3605,7 +3603,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CBC6B76-1F00-43AE-A2F5-6B4E65D9211A}">
-  <dimension ref="A1:R25"/>
+  <dimension ref="A1:R26"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36.75" style="4" bestFit="1" customWidth="1"/>
@@ -5015,6 +5013,62 @@
         <v>38</v>
       </c>
     </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A26" s="21" t="s">
+        <v>192</v>
+      </c>
+      <c r="B26" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="C26" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="D26" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="E26" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="F26" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="G26" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="H26" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="I26" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="J26" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="K26" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="L26" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="M26" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="N26" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="O26" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="P26" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="Q26" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="R26" s="17" t="s">
+        <v>329</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5024,7 +5078,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DCC95B3-8AEE-4FF3-AF94-B2FE3D8B0AED}">
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:R26"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36.75" style="4" bestFit="1" customWidth="1"/>
@@ -5463,7 +5517,7 @@
       </c>
       <c r="I16" s="9"/>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>29</v>
       </c>
@@ -5490,7 +5544,7 @@
       </c>
       <c r="I17" s="9"/>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
         <v>66</v>
       </c>
@@ -5517,7 +5571,7 @@
       </c>
       <c r="I18" s="9"/>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
         <v>58</v>
       </c>
@@ -5544,7 +5598,7 @@
       </c>
       <c r="I19" s="9"/>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
         <v>59</v>
       </c>
@@ -5571,7 +5625,7 @@
       </c>
       <c r="I20" s="9"/>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
         <v>30</v>
       </c>
@@ -5598,7 +5652,7 @@
       </c>
       <c r="I21" s="9"/>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
         <v>60</v>
       </c>
@@ -5625,7 +5679,7 @@
       </c>
       <c r="I22" s="9"/>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
         <v>31</v>
       </c>
@@ -5652,7 +5706,7 @@
       </c>
       <c r="I23" s="9"/>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
         <v>32</v>
       </c>
@@ -5679,7 +5733,7 @@
       </c>
       <c r="I24" s="9"/>
     </row>
-    <row r="25" spans="1:9" ht="33" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:18" ht="33" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
         <v>37</v>
       </c>
@@ -5706,14 +5760,41 @@
       </c>
       <c r="I25" s="9"/>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B26" s="11"/>
-      <c r="C26" s="11"/>
-      <c r="D26" s="11"/>
-      <c r="E26" s="11"/>
-      <c r="F26" s="11"/>
-      <c r="G26" s="11"/>
-      <c r="H26" s="11"/>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A26" s="21" t="s">
+        <v>192</v>
+      </c>
+      <c r="B26" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="C26" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="D26" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="E26" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="F26" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="G26" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="H26" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="I26" s="17"/>
+      <c r="J26" s="17"/>
+      <c r="K26" s="17"/>
+      <c r="L26" s="17"/>
+      <c r="M26" s="17"/>
+      <c r="N26" s="17"/>
+      <c r="O26" s="17"/>
+      <c r="P26" s="17"/>
+      <c r="Q26" s="17"/>
+      <c r="R26" s="17"/>
     </row>
   </sheetData>
   <phoneticPr fontId="18" type="noConversion"/>
@@ -5727,13 +5808,13 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F00BE46B-AB82-49CF-AC58-26BD9D33E867}">
-  <dimension ref="A1:N25"/>
+  <dimension ref="A1:N27"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="36.75" style="24" customWidth="1"/>
-    <col min="2" max="8" width="18.125" style="24" customWidth="1"/>
-    <col min="9" max="14" width="18.125" style="23" customWidth="1"/>
-    <col min="15" max="16384" width="9" style="23"/>
+    <col min="1" max="1" width="36.75" style="4" customWidth="1"/>
+    <col min="2" max="8" width="18.125" style="4" customWidth="1"/>
+    <col min="9" max="14" width="18.125" style="3" customWidth="1"/>
+    <col min="15" max="16384" width="9" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -5784,43 +5865,43 @@
       <c r="A2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="25" t="s">
+      <c r="B2" s="23" t="s">
         <v>85</v>
       </c>
-      <c r="C2" s="25" t="s">
+      <c r="C2" s="23" t="s">
         <v>86</v>
       </c>
-      <c r="D2" s="25" t="s">
+      <c r="D2" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="E2" s="25" t="s">
+      <c r="E2" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="F2" s="25" t="s">
+      <c r="F2" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="G2" s="25" t="s">
+      <c r="G2" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="H2" s="25" t="s">
+      <c r="H2" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="I2" s="25" t="s">
+      <c r="I2" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="J2" s="25" t="s">
+      <c r="J2" s="23" t="s">
         <v>90</v>
       </c>
-      <c r="K2" s="25" t="s">
+      <c r="K2" s="23" t="s">
         <v>91</v>
       </c>
-      <c r="L2" s="25" t="s">
+      <c r="L2" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="M2" s="25" t="s">
+      <c r="M2" s="23" t="s">
         <v>90</v>
       </c>
-      <c r="N2" s="25" t="s">
+      <c r="N2" s="23" t="s">
         <v>91</v>
       </c>
     </row>
@@ -5828,43 +5909,43 @@
       <c r="A3" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="25" t="s">
+      <c r="B3" s="23" t="s">
         <v>92</v>
       </c>
-      <c r="C3" s="25" t="s">
+      <c r="C3" s="23" t="s">
         <v>92</v>
       </c>
-      <c r="D3" s="25" t="s">
+      <c r="D3" s="23" t="s">
         <v>93</v>
       </c>
-      <c r="E3" s="25" t="s">
+      <c r="E3" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="F3" s="25" t="s">
+      <c r="F3" s="23" t="s">
         <v>92</v>
       </c>
-      <c r="G3" s="25" t="s">
+      <c r="G3" s="23" t="s">
         <v>93</v>
       </c>
-      <c r="H3" s="25" t="s">
+      <c r="H3" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="I3" s="25" t="s">
+      <c r="I3" s="23" t="s">
         <v>95</v>
       </c>
-      <c r="J3" s="25" t="s">
+      <c r="J3" s="23" t="s">
         <v>96</v>
       </c>
-      <c r="K3" s="25" t="s">
+      <c r="K3" s="23" t="s">
         <v>97</v>
       </c>
-      <c r="L3" s="25" t="s">
+      <c r="L3" s="23" t="s">
         <v>95</v>
       </c>
-      <c r="M3" s="25" t="s">
+      <c r="M3" s="23" t="s">
         <v>96</v>
       </c>
-      <c r="N3" s="25" t="s">
+      <c r="N3" s="23" t="s">
         <v>97</v>
       </c>
     </row>
@@ -5872,43 +5953,43 @@
       <c r="A4" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="25" t="s">
+      <c r="B4" s="23" t="s">
         <v>98</v>
       </c>
-      <c r="C4" s="25" t="s">
+      <c r="C4" s="23" t="s">
         <v>99</v>
       </c>
-      <c r="D4" s="25" t="s">
+      <c r="D4" s="23" t="s">
         <v>99</v>
       </c>
-      <c r="E4" s="25" t="s">
+      <c r="E4" s="23" t="s">
         <v>99</v>
       </c>
-      <c r="F4" s="25" t="s">
+      <c r="F4" s="23" t="s">
         <v>100</v>
       </c>
-      <c r="G4" s="25" t="s">
+      <c r="G4" s="23" t="s">
         <v>100</v>
       </c>
-      <c r="H4" s="25" t="s">
+      <c r="H4" s="23" t="s">
         <v>100</v>
       </c>
-      <c r="I4" s="25" t="s">
+      <c r="I4" s="23" t="s">
         <v>101</v>
       </c>
-      <c r="J4" s="25" t="s">
+      <c r="J4" s="23" t="s">
         <v>101</v>
       </c>
-      <c r="K4" s="25" t="s">
+      <c r="K4" s="23" t="s">
         <v>101</v>
       </c>
-      <c r="L4" s="25" t="s">
+      <c r="L4" s="23" t="s">
         <v>101</v>
       </c>
-      <c r="M4" s="25" t="s">
+      <c r="M4" s="23" t="s">
         <v>101</v>
       </c>
-      <c r="N4" s="25" t="s">
+      <c r="N4" s="23" t="s">
         <v>101</v>
       </c>
     </row>
@@ -5916,43 +5997,43 @@
       <c r="A5" s="1" t="s">
         <v>307</v>
       </c>
-      <c r="B5" s="25" t="s">
+      <c r="B5" s="23" t="s">
         <v>308</v>
       </c>
-      <c r="C5" s="25" t="s">
+      <c r="C5" s="23" t="s">
         <v>309</v>
       </c>
-      <c r="D5" s="25" t="s">
+      <c r="D5" s="23" t="s">
         <v>310</v>
       </c>
-      <c r="E5" s="25" t="s">
+      <c r="E5" s="23" t="s">
         <v>311</v>
       </c>
-      <c r="F5" s="25" t="s">
+      <c r="F5" s="23" t="s">
         <v>312</v>
       </c>
-      <c r="G5" s="25" t="s">
+      <c r="G5" s="23" t="s">
         <v>313</v>
       </c>
-      <c r="H5" s="25" t="s">
+      <c r="H5" s="23" t="s">
         <v>314</v>
       </c>
-      <c r="I5" s="25" t="s">
+      <c r="I5" s="23" t="s">
         <v>107</v>
       </c>
-      <c r="J5" s="25" t="s">
+      <c r="J5" s="23" t="s">
         <v>109</v>
       </c>
-      <c r="K5" s="25" t="s">
+      <c r="K5" s="23" t="s">
         <v>109</v>
       </c>
-      <c r="L5" s="25" t="s">
+      <c r="L5" s="23" t="s">
         <v>107</v>
       </c>
-      <c r="M5" s="25" t="s">
+      <c r="M5" s="23" t="s">
         <v>109</v>
       </c>
-      <c r="N5" s="25" t="s">
+      <c r="N5" s="23" t="s">
         <v>109</v>
       </c>
     </row>
@@ -5960,43 +6041,43 @@
       <c r="A6" s="1" t="s">
         <v>315</v>
       </c>
-      <c r="B6" s="25" t="s">
+      <c r="B6" s="23" t="s">
         <v>316</v>
       </c>
-      <c r="C6" s="25" t="s">
+      <c r="C6" s="23" t="s">
         <v>317</v>
       </c>
-      <c r="D6" s="25" t="s">
+      <c r="D6" s="23" t="s">
         <v>317</v>
       </c>
-      <c r="E6" s="25" t="s">
+      <c r="E6" s="23" t="s">
         <v>317</v>
       </c>
-      <c r="F6" s="25" t="s">
+      <c r="F6" s="23" t="s">
         <v>317</v>
       </c>
-      <c r="G6" s="25" t="s">
+      <c r="G6" s="23" t="s">
         <v>317</v>
       </c>
-      <c r="H6" s="25" t="s">
+      <c r="H6" s="23" t="s">
         <v>317</v>
       </c>
-      <c r="I6" s="25" t="s">
+      <c r="I6" s="23" t="s">
         <v>111</v>
       </c>
-      <c r="J6" s="25" t="s">
+      <c r="J6" s="23" t="s">
         <v>111</v>
       </c>
-      <c r="K6" s="25" t="s">
+      <c r="K6" s="23" t="s">
         <v>91</v>
       </c>
-      <c r="L6" s="25" t="s">
+      <c r="L6" s="23" t="s">
         <v>111</v>
       </c>
-      <c r="M6" s="25" t="s">
+      <c r="M6" s="23" t="s">
         <v>111</v>
       </c>
-      <c r="N6" s="25" t="s">
+      <c r="N6" s="23" t="s">
         <v>91</v>
       </c>
     </row>
@@ -6004,43 +6085,43 @@
       <c r="A7" s="1" t="s">
         <v>318</v>
       </c>
-      <c r="B7" s="25" t="s">
+      <c r="B7" s="23" t="s">
         <v>112</v>
       </c>
-      <c r="C7" s="25" t="s">
+      <c r="C7" s="23" t="s">
         <v>113</v>
       </c>
-      <c r="D7" s="25" t="s">
+      <c r="D7" s="23" t="s">
         <v>113</v>
       </c>
-      <c r="E7" s="25" t="s">
+      <c r="E7" s="23" t="s">
         <v>113</v>
       </c>
-      <c r="F7" s="25" t="s">
+      <c r="F7" s="23" t="s">
         <v>114</v>
       </c>
-      <c r="G7" s="25" t="s">
+      <c r="G7" s="23" t="s">
         <v>114</v>
       </c>
-      <c r="H7" s="25" t="s">
+      <c r="H7" s="23" t="s">
         <v>114</v>
       </c>
-      <c r="I7" s="25" t="s">
+      <c r="I7" s="23" t="s">
         <v>115</v>
       </c>
-      <c r="J7" s="25" t="s">
+      <c r="J7" s="23" t="s">
         <v>115</v>
       </c>
-      <c r="K7" s="25" t="s">
+      <c r="K7" s="23" t="s">
         <v>115</v>
       </c>
-      <c r="L7" s="25" t="s">
+      <c r="L7" s="23" t="s">
         <v>115</v>
       </c>
-      <c r="M7" s="25" t="s">
+      <c r="M7" s="23" t="s">
         <v>115</v>
       </c>
-      <c r="N7" s="25" t="s">
+      <c r="N7" s="23" t="s">
         <v>115</v>
       </c>
     </row>
@@ -6048,43 +6129,43 @@
       <c r="A8" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="25" t="s">
+      <c r="B8" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="C8" s="25" t="s">
+      <c r="C8" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="D8" s="25" t="s">
+      <c r="D8" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="E8" s="25" t="s">
+      <c r="E8" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="F8" s="25" t="s">
+      <c r="F8" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="G8" s="25" t="s">
+      <c r="G8" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="H8" s="25" t="s">
+      <c r="H8" s="23" t="s">
         <v>42</v>
       </c>
-      <c r="I8" s="25" t="s">
+      <c r="I8" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="J8" s="25" t="s">
+      <c r="J8" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="K8" s="25" t="s">
+      <c r="K8" s="23" t="s">
         <v>44</v>
       </c>
-      <c r="L8" s="25" t="s">
+      <c r="L8" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="M8" s="25" t="s">
+      <c r="M8" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="N8" s="25" t="s">
+      <c r="N8" s="23" t="s">
         <v>44</v>
       </c>
     </row>
@@ -6092,43 +6173,43 @@
       <c r="A9" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="25" t="s">
+      <c r="B9" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="C9" s="25" t="s">
+      <c r="C9" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="D9" s="25" t="s">
+      <c r="D9" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="E9" s="25" t="s">
+      <c r="E9" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="F9" s="25" t="s">
+      <c r="F9" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="G9" s="25" t="s">
+      <c r="G9" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="H9" s="25" t="s">
+      <c r="H9" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="I9" s="25" t="s">
+      <c r="I9" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="J9" s="25" t="s">
+      <c r="J9" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="K9" s="25" t="s">
+      <c r="K9" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="L9" s="25" t="s">
+      <c r="L9" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="M9" s="25" t="s">
+      <c r="M9" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="N9" s="25" t="s">
+      <c r="N9" s="23" t="s">
         <v>40</v>
       </c>
     </row>
@@ -6136,43 +6217,43 @@
       <c r="A10" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B10" s="25" t="s">
+      <c r="B10" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="C10" s="25" t="s">
+      <c r="C10" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="D10" s="25" t="s">
+      <c r="D10" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="E10" s="25" t="s">
+      <c r="E10" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="F10" s="25" t="s">
+      <c r="F10" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="G10" s="25" t="s">
+      <c r="G10" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="H10" s="25" t="s">
+      <c r="H10" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="I10" s="25" t="s">
+      <c r="I10" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="J10" s="25" t="s">
+      <c r="J10" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="K10" s="25" t="s">
+      <c r="K10" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="L10" s="25" t="s">
+      <c r="L10" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="M10" s="25" t="s">
+      <c r="M10" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="N10" s="25" t="s">
+      <c r="N10" s="23" t="s">
         <v>40</v>
       </c>
     </row>
@@ -6180,43 +6261,43 @@
       <c r="A11" s="1" t="s">
         <v>319</v>
       </c>
-      <c r="B11" s="25" t="s">
+      <c r="B11" s="23" t="s">
         <v>117</v>
       </c>
-      <c r="C11" s="25" t="s">
+      <c r="C11" s="23" t="s">
         <v>121</v>
       </c>
-      <c r="D11" s="25" t="s">
+      <c r="D11" s="23" t="s">
         <v>121</v>
       </c>
-      <c r="E11" s="25" t="s">
+      <c r="E11" s="23" t="s">
         <v>121</v>
       </c>
-      <c r="F11" s="25" t="s">
+      <c r="F11" s="23" t="s">
         <v>118</v>
       </c>
-      <c r="G11" s="25" t="s">
+      <c r="G11" s="23" t="s">
         <v>118</v>
       </c>
-      <c r="H11" s="25" t="s">
+      <c r="H11" s="23" t="s">
         <v>118</v>
       </c>
-      <c r="I11" s="25" t="s">
+      <c r="I11" s="23" t="s">
         <v>119</v>
       </c>
-      <c r="J11" s="25" t="s">
+      <c r="J11" s="23" t="s">
         <v>119</v>
       </c>
-      <c r="K11" s="25" t="s">
+      <c r="K11" s="23" t="s">
         <v>119</v>
       </c>
-      <c r="L11" s="25" t="s">
+      <c r="L11" s="23" t="s">
         <v>120</v>
       </c>
-      <c r="M11" s="25" t="s">
+      <c r="M11" s="23" t="s">
         <v>120</v>
       </c>
-      <c r="N11" s="25" t="s">
+      <c r="N11" s="23" t="s">
         <v>120</v>
       </c>
     </row>
@@ -6224,43 +6305,43 @@
       <c r="A12" s="1" t="s">
         <v>320</v>
       </c>
-      <c r="B12" s="25" t="s">
+      <c r="B12" s="23" t="s">
         <v>187</v>
       </c>
-      <c r="C12" s="25" t="s">
+      <c r="C12" s="23" t="s">
         <v>188</v>
       </c>
-      <c r="D12" s="25" t="s">
+      <c r="D12" s="23" t="s">
         <v>188</v>
       </c>
-      <c r="E12" s="25" t="s">
+      <c r="E12" s="23" t="s">
         <v>188</v>
       </c>
-      <c r="F12" s="25" t="s">
+      <c r="F12" s="23" t="s">
         <v>119</v>
       </c>
-      <c r="G12" s="25" t="s">
+      <c r="G12" s="23" t="s">
         <v>119</v>
       </c>
-      <c r="H12" s="25" t="s">
+      <c r="H12" s="23" t="s">
         <v>119</v>
       </c>
-      <c r="I12" s="25" t="s">
+      <c r="I12" s="23" t="s">
         <v>123</v>
       </c>
-      <c r="J12" s="25" t="s">
+      <c r="J12" s="23" t="s">
         <v>123</v>
       </c>
-      <c r="K12" s="25" t="s">
+      <c r="K12" s="23" t="s">
         <v>123</v>
       </c>
-      <c r="L12" s="25" t="s">
+      <c r="L12" s="23" t="s">
         <v>124</v>
       </c>
-      <c r="M12" s="25" t="s">
+      <c r="M12" s="23" t="s">
         <v>124</v>
       </c>
-      <c r="N12" s="25" t="s">
+      <c r="N12" s="23" t="s">
         <v>124</v>
       </c>
     </row>
@@ -6268,43 +6349,43 @@
       <c r="A13" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="B13" s="25" t="s">
+      <c r="B13" s="23" t="s">
         <v>125</v>
       </c>
-      <c r="C13" s="25" t="s">
+      <c r="C13" s="23" t="s">
         <v>126</v>
       </c>
-      <c r="D13" s="25" t="s">
+      <c r="D13" s="23" t="s">
         <v>126</v>
       </c>
-      <c r="E13" s="25" t="s">
+      <c r="E13" s="23" t="s">
         <v>126</v>
       </c>
-      <c r="F13" s="25" t="s">
+      <c r="F13" s="23" t="s">
         <v>127</v>
       </c>
-      <c r="G13" s="25" t="s">
+      <c r="G13" s="23" t="s">
         <v>127</v>
       </c>
-      <c r="H13" s="25" t="s">
+      <c r="H13" s="23" t="s">
         <v>127</v>
       </c>
-      <c r="I13" s="25" t="s">
+      <c r="I13" s="23" t="s">
         <v>128</v>
       </c>
-      <c r="J13" s="25" t="s">
+      <c r="J13" s="23" t="s">
         <v>128</v>
       </c>
-      <c r="K13" s="25" t="s">
+      <c r="K13" s="23" t="s">
         <v>128</v>
       </c>
-      <c r="L13" s="25" t="s">
+      <c r="L13" s="23" t="s">
         <v>129</v>
       </c>
-      <c r="M13" s="25" t="s">
+      <c r="M13" s="23" t="s">
         <v>129</v>
       </c>
-      <c r="N13" s="25" t="s">
+      <c r="N13" s="23" t="s">
         <v>129</v>
       </c>
     </row>
@@ -6312,43 +6393,43 @@
       <c r="A14" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="B14" s="25" t="s">
+      <c r="B14" s="23" t="s">
         <v>130</v>
       </c>
-      <c r="C14" s="25" t="s">
+      <c r="C14" s="23" t="s">
         <v>131</v>
       </c>
-      <c r="D14" s="25" t="s">
+      <c r="D14" s="23" t="s">
         <v>131</v>
       </c>
-      <c r="E14" s="25" t="s">
+      <c r="E14" s="23" t="s">
         <v>131</v>
       </c>
-      <c r="F14" s="25" t="s">
+      <c r="F14" s="23" t="s">
         <v>132</v>
       </c>
-      <c r="G14" s="25" t="s">
+      <c r="G14" s="23" t="s">
         <v>132</v>
       </c>
-      <c r="H14" s="25" t="s">
+      <c r="H14" s="23" t="s">
         <v>132</v>
       </c>
-      <c r="I14" s="25" t="s">
+      <c r="I14" s="23" t="s">
         <v>133</v>
       </c>
-      <c r="J14" s="25" t="s">
+      <c r="J14" s="23" t="s">
         <v>133</v>
       </c>
-      <c r="K14" s="25" t="s">
+      <c r="K14" s="23" t="s">
         <v>133</v>
       </c>
-      <c r="L14" s="25" t="s">
+      <c r="L14" s="23" t="s">
         <v>133</v>
       </c>
-      <c r="M14" s="25" t="s">
+      <c r="M14" s="23" t="s">
         <v>133</v>
       </c>
-      <c r="N14" s="25" t="s">
+      <c r="N14" s="23" t="s">
         <v>133</v>
       </c>
     </row>
@@ -6356,25 +6437,25 @@
       <c r="A15" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B15" s="25" t="s">
+      <c r="B15" s="23" t="s">
         <v>328</v>
       </c>
-      <c r="C15" s="25" t="s">
+      <c r="C15" s="23" t="s">
         <v>328</v>
       </c>
-      <c r="D15" s="25" t="s">
+      <c r="D15" s="23" t="s">
         <v>328</v>
       </c>
-      <c r="E15" s="25" t="s">
+      <c r="E15" s="23" t="s">
         <v>328</v>
       </c>
-      <c r="F15" s="25" t="s">
+      <c r="F15" s="23" t="s">
         <v>328</v>
       </c>
-      <c r="G15" s="25" t="s">
+      <c r="G15" s="23" t="s">
         <v>328</v>
       </c>
-      <c r="H15" s="25" t="s">
+      <c r="H15" s="23" t="s">
         <v>328</v>
       </c>
       <c r="I15" s="7" t="s">
@@ -6400,43 +6481,43 @@
       <c r="A16" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B16" s="25" t="s">
+      <c r="B16" s="23" t="s">
         <v>255</v>
       </c>
-      <c r="C16" s="25" t="s">
+      <c r="C16" s="23" t="s">
         <v>136</v>
       </c>
-      <c r="D16" s="25" t="s">
+      <c r="D16" s="23" t="s">
         <v>321</v>
       </c>
-      <c r="E16" s="25" t="s">
+      <c r="E16" s="23" t="s">
         <v>322</v>
       </c>
-      <c r="F16" s="25" t="s">
+      <c r="F16" s="23" t="s">
         <v>139</v>
       </c>
-      <c r="G16" s="25" t="s">
+      <c r="G16" s="23" t="s">
         <v>322</v>
       </c>
-      <c r="H16" s="25" t="s">
+      <c r="H16" s="23" t="s">
         <v>323</v>
       </c>
-      <c r="I16" s="25" t="s">
+      <c r="I16" s="23" t="s">
         <v>140</v>
       </c>
-      <c r="J16" s="25" t="s">
+      <c r="J16" s="23" t="s">
         <v>141</v>
       </c>
-      <c r="K16" s="25" t="s">
+      <c r="K16" s="23" t="s">
         <v>142</v>
       </c>
-      <c r="L16" s="25" t="s">
+      <c r="L16" s="23" t="s">
         <v>143</v>
       </c>
-      <c r="M16" s="25" t="s">
+      <c r="M16" s="23" t="s">
         <v>144</v>
       </c>
-      <c r="N16" s="25" t="s">
+      <c r="N16" s="23" t="s">
         <v>145</v>
       </c>
     </row>
@@ -6532,43 +6613,43 @@
       <c r="A19" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="B19" s="25" t="s">
+      <c r="B19" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="C19" s="25" t="s">
+      <c r="C19" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="D19" s="25" t="s">
+      <c r="D19" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="E19" s="25" t="s">
+      <c r="E19" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="F19" s="25" t="s">
+      <c r="F19" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="G19" s="25" t="s">
+      <c r="G19" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="H19" s="25" t="s">
+      <c r="H19" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="I19" s="25" t="s">
+      <c r="I19" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="J19" s="25" t="s">
+      <c r="J19" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="K19" s="25" t="s">
+      <c r="K19" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="L19" s="25" t="s">
+      <c r="L19" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="M19" s="25" t="s">
+      <c r="M19" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="N19" s="25" t="s">
+      <c r="N19" s="23" t="s">
         <v>48</v>
       </c>
     </row>
@@ -6576,43 +6657,43 @@
       <c r="A20" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="B20" s="25" t="s">
+      <c r="B20" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="C20" s="25" t="s">
+      <c r="C20" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="D20" s="25" t="s">
+      <c r="D20" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="E20" s="25" t="s">
+      <c r="E20" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="F20" s="25" t="s">
+      <c r="F20" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="G20" s="25" t="s">
+      <c r="G20" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="H20" s="25" t="s">
+      <c r="H20" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="I20" s="25" t="s">
+      <c r="I20" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="J20" s="25" t="s">
+      <c r="J20" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="K20" s="25" t="s">
+      <c r="K20" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="L20" s="25" t="s">
+      <c r="L20" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="M20" s="25" t="s">
+      <c r="M20" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="N20" s="25" t="s">
+      <c r="N20" s="23" t="s">
         <v>53</v>
       </c>
     </row>
@@ -6620,43 +6701,43 @@
       <c r="A21" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B21" s="25" t="s">
+      <c r="B21" s="23" t="s">
         <v>148</v>
       </c>
-      <c r="C21" s="25" t="s">
+      <c r="C21" s="23" t="s">
         <v>149</v>
       </c>
-      <c r="D21" s="25" t="s">
+      <c r="D21" s="23" t="s">
         <v>149</v>
       </c>
-      <c r="E21" s="25" t="s">
+      <c r="E21" s="23" t="s">
         <v>149</v>
       </c>
-      <c r="F21" s="25" t="s">
+      <c r="F21" s="23" t="s">
         <v>149</v>
       </c>
-      <c r="G21" s="25" t="s">
+      <c r="G21" s="23" t="s">
         <v>149</v>
       </c>
-      <c r="H21" s="25" t="s">
+      <c r="H21" s="23" t="s">
         <v>149</v>
       </c>
-      <c r="I21" s="25" t="s">
+      <c r="I21" s="23" t="s">
         <v>150</v>
       </c>
-      <c r="J21" s="25" t="s">
+      <c r="J21" s="23" t="s">
         <v>150</v>
       </c>
-      <c r="K21" s="25" t="s">
+      <c r="K21" s="23" t="s">
         <v>150</v>
       </c>
-      <c r="L21" s="25" t="s">
+      <c r="L21" s="23" t="s">
         <v>95</v>
       </c>
-      <c r="M21" s="25" t="s">
+      <c r="M21" s="23" t="s">
         <v>95</v>
       </c>
-      <c r="N21" s="25" t="s">
+      <c r="N21" s="23" t="s">
         <v>95</v>
       </c>
     </row>
@@ -6664,43 +6745,43 @@
       <c r="A22" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="B22" s="25" t="s">
+      <c r="B22" s="23" t="s">
         <v>54</v>
       </c>
-      <c r="C22" s="25" t="s">
+      <c r="C22" s="23" t="s">
         <v>54</v>
       </c>
-      <c r="D22" s="25" t="s">
+      <c r="D22" s="23" t="s">
         <v>54</v>
       </c>
-      <c r="E22" s="25" t="s">
+      <c r="E22" s="23" t="s">
         <v>54</v>
       </c>
-      <c r="F22" s="25" t="s">
+      <c r="F22" s="23" t="s">
         <v>54</v>
       </c>
-      <c r="G22" s="25" t="s">
+      <c r="G22" s="23" t="s">
         <v>54</v>
       </c>
-      <c r="H22" s="25" t="s">
+      <c r="H22" s="23" t="s">
         <v>54</v>
       </c>
-      <c r="I22" s="25" t="s">
+      <c r="I22" s="23" t="s">
         <v>54</v>
       </c>
-      <c r="J22" s="25" t="s">
+      <c r="J22" s="23" t="s">
         <v>54</v>
       </c>
-      <c r="K22" s="25" t="s">
+      <c r="K22" s="23" t="s">
         <v>54</v>
       </c>
-      <c r="L22" s="25" t="s">
+      <c r="L22" s="23" t="s">
         <v>54</v>
       </c>
-      <c r="M22" s="25" t="s">
+      <c r="M22" s="23" t="s">
         <v>54</v>
       </c>
-      <c r="N22" s="25" t="s">
+      <c r="N22" s="23" t="s">
         <v>54</v>
       </c>
     </row>
@@ -6708,43 +6789,43 @@
       <c r="A23" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B23" s="25" t="s">
+      <c r="B23" s="23" t="s">
         <v>324</v>
       </c>
-      <c r="C23" s="25" t="s">
+      <c r="C23" s="23" t="s">
         <v>157</v>
       </c>
-      <c r="D23" s="25" t="s">
+      <c r="D23" s="23" t="s">
         <v>325</v>
       </c>
-      <c r="E23" s="25" t="s">
+      <c r="E23" s="23" t="s">
         <v>326</v>
       </c>
-      <c r="F23" s="25" t="s">
+      <c r="F23" s="23" t="s">
         <v>152</v>
       </c>
-      <c r="G23" s="25" t="s">
+      <c r="G23" s="23" t="s">
         <v>327</v>
       </c>
-      <c r="H23" s="25" t="s">
+      <c r="H23" s="23" t="s">
         <v>154</v>
       </c>
-      <c r="I23" s="25" t="s">
+      <c r="I23" s="23" t="s">
         <v>156</v>
       </c>
-      <c r="J23" s="25" t="s">
+      <c r="J23" s="23" t="s">
         <v>157</v>
       </c>
-      <c r="K23" s="25" t="s">
+      <c r="K23" s="23" t="s">
         <v>151</v>
       </c>
-      <c r="L23" s="25" t="s">
+      <c r="L23" s="23" t="s">
         <v>158</v>
       </c>
-      <c r="M23" s="25" t="s">
+      <c r="M23" s="23" t="s">
         <v>156</v>
       </c>
-      <c r="N23" s="25" t="s">
+      <c r="N23" s="23" t="s">
         <v>153</v>
       </c>
     </row>
@@ -6752,43 +6833,43 @@
       <c r="A24" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B24" s="25" t="s">
+      <c r="B24" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="C24" s="25" t="s">
+      <c r="C24" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="D24" s="25" t="s">
+      <c r="D24" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="E24" s="25" t="s">
+      <c r="E24" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="F24" s="25" t="s">
+      <c r="F24" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="G24" s="25" t="s">
+      <c r="G24" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="H24" s="25" t="s">
+      <c r="H24" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="I24" s="25" t="s">
+      <c r="I24" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="J24" s="25" t="s">
+      <c r="J24" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="K24" s="25" t="s">
+      <c r="K24" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="L24" s="25" t="s">
+      <c r="L24" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="M24" s="25" t="s">
+      <c r="M24" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="N24" s="25" t="s">
+      <c r="N24" s="23" t="s">
         <v>35</v>
       </c>
     </row>
@@ -6796,45 +6877,98 @@
       <c r="A25" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B25" s="25" t="s">
+      <c r="B25" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="C25" s="25" t="s">
+      <c r="C25" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="D25" s="25" t="s">
+      <c r="D25" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="E25" s="25" t="s">
+      <c r="E25" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="F25" s="25" t="s">
+      <c r="F25" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="G25" s="25" t="s">
+      <c r="G25" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="H25" s="25" t="s">
+      <c r="H25" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="I25" s="25" t="s">
+      <c r="I25" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="J25" s="25" t="s">
+      <c r="J25" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="K25" s="25" t="s">
+      <c r="K25" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="L25" s="25" t="s">
+      <c r="L25" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="M25" s="25" t="s">
+      <c r="M25" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="N25" s="25" t="s">
+      <c r="N25" s="23" t="s">
         <v>39</v>
       </c>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A26" s="21" t="s">
+        <v>192</v>
+      </c>
+      <c r="B26" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="C26" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="D26" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="E26" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="F26" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="G26" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="H26" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="I26" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="J26" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="K26" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="L26" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="M26" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="N26" s="17" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="H27" s="17"/>
+      <c r="I27" s="17"/>
+      <c r="J27" s="17"/>
+      <c r="K27" s="17"/>
+      <c r="L27" s="17"/>
+      <c r="M27" s="17"/>
+      <c r="N27" s="17"/>
     </row>
   </sheetData>
   <phoneticPr fontId="18" type="noConversion"/>

</xml_diff>